<commit_message>
auto: snapshot 2026-07-27 05:00:09
</commit_message>
<xml_diff>
--- a/clan_110.xlsx
+++ b/clan_110.xlsx
@@ -8,6 +8,7 @@
   </bookViews>
   <sheets>
     <sheet name="2026-07-26" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="2026-07-27" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -509,4 +510,82 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="19" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Zanasis eSports (110) | S62</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Day Points</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-07-27 13:00:09</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>Edward_Newgate</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
auto: snapshot 2026-07-28 05:00:11
</commit_message>
<xml_diff>
--- a/clan_110.xlsx
+++ b/clan_110.xlsx
@@ -9,6 +9,7 @@
   <sheets>
     <sheet name="2026-07-26" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="2026-07-27" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="2026-07-28" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -588,4 +589,82 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="19" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Zanasis eSports (110) | S62</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Day Points</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-07-28 13:00:10</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>Edward_Newgate</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
auto: snapshot 2026-07-29 05:00:13
</commit_message>
<xml_diff>
--- a/clan_110.xlsx
+++ b/clan_110.xlsx
@@ -10,6 +10,7 @@
     <sheet name="2026-07-26" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="2026-07-27" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="2026-07-28" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="2026-07-29" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -667,4 +668,82 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="19" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Zanasis eSports (110) | S62</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Day Points</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-07-29 13:00:12</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>Edward_Newgate</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
auto: snapshot 2026-07-30 05:00:21
</commit_message>
<xml_diff>
--- a/clan_110.xlsx
+++ b/clan_110.xlsx
@@ -11,6 +11,7 @@
     <sheet name="2026-07-27" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="2026-07-28" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="2026-07-29" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="2026-07-30" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -746,4 +747,82 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="19" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Zanasis eSports (110) | S62</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Day Points</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-07-30 13:00:21</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>Edward_Newgate</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
auto: snapshot 2026-07-31 05:00:22
</commit_message>
<xml_diff>
--- a/clan_110.xlsx
+++ b/clan_110.xlsx
@@ -12,6 +12,7 @@
     <sheet name="2026-07-28" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="2026-07-29" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="2026-07-30" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="2026-07-31" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -825,4 +826,82 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="19" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Zanasis eSports (110) | S62</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Day Points</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-07-31 13:00:22</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>Edward_Newgate</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
auto: snapshot 2026-08-01 05:00:34
</commit_message>
<xml_diff>
--- a/clan_110.xlsx
+++ b/clan_110.xlsx
@@ -13,6 +13,7 @@
     <sheet name="2026-07-29" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="2026-07-30" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="2026-07-31" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="2026-08-01" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -904,4 +905,82 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="19" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Zanasis eSports (110) | S62</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Day Points</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-08-01 13:00:34</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>Edward_Newgate</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
auto: snapshot 2026-08-02 05:01:44
</commit_message>
<xml_diff>
--- a/clan_110.xlsx
+++ b/clan_110.xlsx
@@ -14,6 +14,7 @@
     <sheet name="2026-07-30" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="2026-07-31" sheetId="6" state="visible" r:id="rId6"/>
     <sheet name="2026-08-01" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="2026-08-02" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -983,4 +984,82 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="19" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Zanasis eSports (110) | S62</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Day Points</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-08-02 13:01:44</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>Edward_Newgate</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
auto: snapshot 2026-08-03 05:00:14
</commit_message>
<xml_diff>
--- a/clan_110.xlsx
+++ b/clan_110.xlsx
@@ -15,6 +15,7 @@
     <sheet name="2026-07-31" sheetId="6" state="visible" r:id="rId6"/>
     <sheet name="2026-08-01" sheetId="7" state="visible" r:id="rId7"/>
     <sheet name="2026-08-02" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="2026-08-03" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1062,4 +1063,82 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="19" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Zanasis eSports (110) | S62</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Day Points</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-08-03 13:00:14</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>Edward_Newgate</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
auto: snapshot 2026-08-05 05:00:19
</commit_message>
<xml_diff>
--- a/clan_110.xlsx
+++ b/clan_110.xlsx
@@ -17,6 +17,7 @@
     <sheet name="2026-08-02" sheetId="8" state="visible" r:id="rId8"/>
     <sheet name="2026-08-03" sheetId="9" state="visible" r:id="rId9"/>
     <sheet name="2026-08-04" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="2026-08-05" sheetId="11" state="visible" r:id="rId11"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -598,6 +599,84 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="19" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Zanasis eSports (110) | S62</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Day Points</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-08-05 13:00:18</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>Edward_Newgate</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>